<commit_message>
Add configurable skill levels and effects
</commit_message>
<xml_diff>
--- a/Client/Configs/GameConfig/Datas/__tables__.xlsx
+++ b/Client/Configs/GameConfig/Datas/__tables__.xlsx
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="3"/>
   <cols>
     <col width="12" customWidth="1" style="2" min="1" max="1"/>
@@ -1175,222 +1175,262 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="0" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>item.TbItem</t>
         </is>
       </c>
-      <c r="C4" s="0" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="D4" s="0" t="b">
+      <c r="D4" t="b">
         <v>1</v>
       </c>
-      <c r="E4" s="0" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>item.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="0" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>skill.TbSkill</t>
         </is>
       </c>
-      <c r="C5" s="0" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Skill</t>
         </is>
       </c>
-      <c r="D5" s="0" t="b">
+      <c r="D5" t="b">
         <v>1</v>
       </c>
-      <c r="E5" s="0" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>skill.xlsx</t>
         </is>
       </c>
-      <c r="F5" s="0" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="G5" s="0" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>map</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>技能主表：原型阶段优先编辑这里。配置技能ID、显示名、冷却、距离、动画Key，并引用效果和投射物。</t>
+          <t>??????????????ID???????????????????? skill_level.xlsx?</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>常用</t>
+          <t>??</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="0" t="inlineStr">
-        <is>
-          <t>skill.TbSkillEffect</t>
-        </is>
-      </c>
-      <c r="C6" s="0" t="inlineStr">
-        <is>
-          <t>SkillEffect</t>
-        </is>
-      </c>
-      <c r="D6" s="0" t="b">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>skill.TbSkillLevel</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SkillLevel</t>
+        </is>
+      </c>
+      <c r="D6" t="b">
         <v>1</v>
       </c>
-      <c r="E6" s="0" t="inlineStr">
-        <is>
-          <t>skill_effect.xlsx</t>
-        </is>
-      </c>
-      <c r="F6" s="0" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>skill_level.xlsx</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="G6" s="0" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>map</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>高级预留：一个技能多个效果/多个触发阶段时再启用。当前运行时还主要读取 skill.effectId。</t>
+          <t>????????? skillId ??? level ???????????????????</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>预留</t>
+          <t>??</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="0" t="inlineStr">
-        <is>
-          <t>skill.TbEffect</t>
-        </is>
-      </c>
-      <c r="C7" s="0" t="inlineStr">
-        <is>
-          <t>Effect</t>
-        </is>
-      </c>
-      <c r="D7" s="0" t="b">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>skill.TbSkillEffect</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SkillEffect</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
         <v>1</v>
       </c>
-      <c r="E7" s="0" t="inlineStr">
-        <is>
-          <t>effect.xlsx</t>
-        </is>
-      </c>
-      <c r="F7" s="0" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>skill_effect.xlsx</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="G7" s="0" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>map</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>效果表：配置命中后造成什么逻辑效果，例如伤害、治疗、击退、控制、加Buff。</t>
+          <t>????????? skillId + level + order ???? effect?</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>常用</t>
+          <t>??</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="0" t="inlineStr">
-        <is>
-          <t>skill.TbBuff</t>
-        </is>
-      </c>
-      <c r="C8" s="0" t="inlineStr">
-        <is>
-          <t>Buff</t>
-        </is>
-      </c>
-      <c r="D8" s="0" t="b">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>skill.TbEffect</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Effect</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
         <v>1</v>
       </c>
-      <c r="E8" s="0" t="inlineStr">
-        <is>
-          <t>buff.xlsx</t>
-        </is>
-      </c>
-      <c r="F8" s="0" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>effect.xlsx</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="G8" s="0" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>map</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Buff预留表：配置持续效果、减速、眩晕、光环、属性加成等。当前原型可以先不改。</t>
+          <t>?????????????Buff???????</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>预留</t>
+          <t>??</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="0" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>skill.TbBuff</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Buff</t>
+        </is>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>buff.xlsx</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Buff???????????????????????</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>??</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
         <is>
           <t>skill.TbProjectile</t>
         </is>
       </c>
-      <c r="C9" s="0" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Projectile</t>
         </is>
       </c>
-      <c r="D9" s="0" t="b">
+      <c r="D10" t="b">
         <v>1</v>
       </c>
-      <c r="E9" s="0" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>projectile.xlsx</t>
         </is>
       </c>
-      <c r="F9" s="0" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="G9" s="0" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>map</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>投射物表现表：配置技能飞行速度、飞行Prefab、出手特效、命中特效和备用颜色。</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>常用</t>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>??????????????Prefab????????</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>??</t>
         </is>
       </c>
     </row>

</xml_diff>